<commit_message>
WIP: Add SharpPcap/PacketDotNet packages for robust cross-platform PCAP parsing
Co-authored-by: dongnuc <136960214+dongnuc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_run/AnhDThe187386/OverallSummary.xlsx
+++ b/test_run/AnhDThe187386/OverallSummary.xlsx
@@ -34,28 +34,28 @@
     <x:t>TC1</x:t>
   </x:si>
   <x:si>
+    <x:t>PASS</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>TC2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TC3</x:t>
+  </x:si>
+  <x:si>
     <x:t>FAIL</x:t>
   </x:si>
   <x:si>
-    <x:t>Network flows: 2 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TC2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Network flows: 3 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TC3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Network flows: 7 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
+    <x:t>Network flows: 3 FAIL (ALL-OR-NOTHING), 4 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC4</x:t>
   </x:si>
   <x:si>
-    <x:t>Network flows: 11 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
+    <x:t>Network flows: 5 FAIL (ALL-OR-NOTHING), 6 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC5</x:t>
@@ -64,7 +64,7 @@
     <x:t>TC6</x:t>
   </x:si>
   <x:si>
-    <x:t>Network flows: 22 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
+    <x:t>Network flows: 10 FAIL (ALL-OR-NOTHING), 12 PASS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -437,7 +437,7 @@
     <x:col min="2" max="2" width="7.282054" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="11.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.567768" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="45.424911" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:5" s="1" customFormat="1">
@@ -465,7 +465,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>0.5</x:v>
@@ -482,21 +482,21 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
         <x:v>10</x:v>
-      </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="0">
         <x:v>0</x:v>
@@ -513,7 +513,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="0">
         <x:v>0</x:v>
@@ -530,7 +530,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="0">
         <x:v>0</x:v>
@@ -547,7 +547,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C7" s="0">
         <x:v>0</x:v>

</xml_diff>